<commit_message>
Product And Accessories Automation Script
</commit_message>
<xml_diff>
--- a/ZlaataQA/src/test/resources/ImportFile/supplier_template.xlsx
+++ b/ZlaataQA/src/test/resources/ImportFile/supplier_template.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="134">
   <si>
     <t>India</t>
   </si>
@@ -356,6 +356,75 @@
   </si>
   <si>
     <t>7448579832</t>
+  </si>
+  <si>
+    <t>9194_Automation Test Supplier</t>
+  </si>
+  <si>
+    <t>supplier_9194@abc.com</t>
+  </si>
+  <si>
+    <t>8426085322</t>
+  </si>
+  <si>
+    <t>Chris Miller</t>
+  </si>
+  <si>
+    <t>chris.miller9194@abc.com</t>
+  </si>
+  <si>
+    <t>9541110903</t>
+  </si>
+  <si>
+    <t>5750_Automation Test Supplier</t>
+  </si>
+  <si>
+    <t>supplier_5750@abc.com</t>
+  </si>
+  <si>
+    <t>9412671849</t>
+  </si>
+  <si>
+    <t>Taylor Garcia</t>
+  </si>
+  <si>
+    <t>taylor.garcia5750@abc.com</t>
+  </si>
+  <si>
+    <t>7803479551</t>
+  </si>
+  <si>
+    <t>3278_Automation Test Supplier</t>
+  </si>
+  <si>
+    <t>supplier_3278@abc.com</t>
+  </si>
+  <si>
+    <t>9756845733</t>
+  </si>
+  <si>
+    <t>Jordan Garcia</t>
+  </si>
+  <si>
+    <t>jordan.garcia3278@abc.com</t>
+  </si>
+  <si>
+    <t>9745302682</t>
+  </si>
+  <si>
+    <t>2832_Automation Test Supplier</t>
+  </si>
+  <si>
+    <t>supplier_2832@abc.com</t>
+  </si>
+  <si>
+    <t>7388838375</t>
+  </si>
+  <si>
+    <t>morgan.smith2832@abc.com</t>
+  </si>
+  <si>
+    <t>7567475044</t>
   </si>
 </sst>
 </file>
@@ -1171,13 +1240,13 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B3" t="s" s="0">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>62</v>
@@ -1186,13 +1255,13 @@
         <v>1</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="I3" s="0" t="s">
-        <v>110</v>
+        <v>133</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>17</v>

</xml_diff>